<commit_message>
Kindle becomes Sun Warrior's Breath and restores 10% Mana over 10 s
Renamed in design/Ability_Tree.xlsx (ability and scroll) and re-imported; a
mana-over-time buff property; old saves' Kindling Scroll maps to the new id.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NkxcXD4xqQYvGrzBVzDJEX
</commit_message>
<xml_diff>
--- a/design/Ability_Tree.xlsx
+++ b/design/Ability_Tree.xlsx
@@ -166,16 +166,16 @@
     <t xml:space="preserve">F04</t>
   </si>
   <si>
-    <t xml:space="preserve">Kindle</t>
+    <t xml:space="preserve">Sun Warrior's Breath</t>
   </si>
   <si>
     <t xml:space="preserve">Self buff</t>
   </si>
   <si>
-    <t xml:space="preserve">Kindling Scroll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Your next 3 fire abilities deal bonus damage.</t>
+    <t xml:space="preserve">Sun Warrior's Breath Scroll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your next 3 fire abilities deal bonus damage, and you regain 10% of your Mana over 10s.</t>
   </si>
   <si>
     <t xml:space="preserve">Self</t>

</xml_diff>

<commit_message>
Several inputs per timing bar; aimed abilities fire where the cursor points at the end; Quick Shot and Aimed Shot bars
Quick Shot: 2 s, hold 0.25-1.75. Aimed Shot: 4 s, tap then hold. Inputs are
played in order; power is their average, crit only if all are perfect.
Crits now travel with projectiles and delayed hits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/Ability_Tree.xlsx
+++ b/design/Ability_Tree.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloig\Documents\GitHub\Final-Wars\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DAB134A-9CF7-45AF-B5E0-4890F6E20542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4390271-613D-430B-83F8-9052E54E72C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28455" yWindow="4770" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Tiers" sheetId="2" r:id="rId2"/>
     <sheet name="Trees" sheetId="3" r:id="rId3"/>
     <sheet name="Rules &amp; Legend" sheetId="4" r:id="rId4"/>
-    <sheet name="Timing Rules" sheetId="6" r:id="rId5"/>
+    <sheet name="Timing Rules" sheetId="7" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Abilities!$A$1:$T$146</definedName>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2391" uniqueCount="1171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2395" uniqueCount="1175">
   <si>
     <t>ID</t>
   </si>
@@ -3084,18 +3084,6 @@
     <t>No bar: a dash then a strike (dashes have no bar).</t>
   </si>
   <si>
-    <t>Tap 0.30–0.55; Crit 0.40–0.50</t>
-  </si>
-  <si>
-    <t>Bow: quick shot, middle beat.</t>
-  </si>
-  <si>
-    <t>Hold 0.25–1.25</t>
-  </si>
-  <si>
-    <t>Bow: drawing = holding; replaces its 1 s draw. The arrow flies when you let go.</t>
-  </si>
-  <si>
     <t>Tap 0.80–1.10; Crit 0.95–1.05</t>
   </si>
   <si>
@@ -3132,12 +3120,6 @@
     <t>Moving, a stun, an interrupt, or a Targeted target leaving range or line of sight cancels the bar; the cooldown is not spent.</t>
   </si>
   <si>
-    <t>One input per bar</t>
-  </si>
-  <si>
-    <t>For now a bar takes one input: a tap casts the ability at once, a hold casts it when let go. The sheet already accepts several zones per bar (for future complex spells); the game then counts only the first press.</t>
-  </si>
-  <si>
     <t>Who plays them</t>
   </si>
   <si>
@@ -3360,18 +3342,12 @@
     <t>The bar's length in seconds, or 'none' for an ability that has no bar (an instant).</t>
   </si>
   <si>
-    <t>Zones separated by ';', each 'Tap a–b', 'Crit a–b' or 'Hold a–b', in seconds from the bar's start (for example 'Tap 0.35–0.65; Crit 0.45–0.55' or 'Hold 0.75–2.75'). Dots or commas for decimals; '-' or '–' between the numbers.</t>
-  </si>
-  <si>
     <t>Free text: the idea behind the design.</t>
   </si>
   <si>
     <t>After editing</t>
   </si>
   <si>
-    <t>Re-import the sheet (docs/ability-import.md). The import checks that every zone is inside its bar, that holds end 0.2–0.3 s before the bar, that crits sit inside a tap, and that the numbers read; it refuses the file otherwise.</t>
-  </si>
-  <si>
     <t>Tunable values (ask to change them)</t>
   </si>
   <si>
@@ -3540,9 +3516,6 @@
     <t>100%</t>
   </si>
   <si>
-    <t>Above the bar for 0.8 s: Miss, Good or Perfect!; a hold adds its accuracy, e.g. Good 88%.</t>
-  </si>
-  <si>
     <t>Hold! is shown while holding and the held part turns light blue. Past the zone the label turns red (Let go!) and the extra time is drawn red; so is a press before the zone.</t>
   </si>
   <si>
@@ -3556,6 +3529,45 @@
   </si>
   <si>
     <t>+50%</t>
+  </si>
+  <si>
+    <t>Hold 0.25–1.75</t>
+  </si>
+  <si>
+    <t>Designer's bar: hold 1.5 s at the end, ending 0.25 s before the bar. The arrow flies where the cursor points when you let go.</t>
+  </si>
+  <si>
+    <t>Tap 0.20–0.60; Crit 0.35–0.45; Hold 1.00–3.75</t>
+  </si>
+  <si>
+    <t>Designer's bar: a tap at the start (nock), then hold to the end (draw), ending 0.25 s before the bar. Replaces its 1 s draw. Fires where the cursor points when you let go.</t>
+  </si>
+  <si>
+    <t>Inputs in order</t>
+  </si>
+  <si>
+    <t>A bar may ask for several inputs (taps and holds), played in order, one press each (Aimed Shot: a tap, then a hold). A press goes to the next input whose window isn't over; an input skipped or never played counts as a miss. The ability goes off when the last input is played (a tap at once, a hold when let go), or when the bar ends.</t>
+  </si>
+  <si>
+    <t>Aimed abilities</t>
+  </si>
+  <si>
+    <t>Skillshots and ground abilities with a bar start their bar as soon as the key is pressed; the affected tiles follow the cursor during the bar, and the ability fires where the cursor points at the last input (a ground target beyond range is pulled back to the edge of the range). Aimed abilities without a bar (Flame Dash, Raise Pillar, Earth Wall) still aim first: hold the key, release to cast.</t>
+  </si>
+  <si>
+    <t>Several inputs</t>
+  </si>
+  <si>
+    <t>The bar's power is the average of its inputs' powers (a tap 70% or 100%, a hold 70% to 100% by accuracy). Critical success only if every input is perfect (a yellow tap, a 95%+ hold); a miss only if every input is a miss; otherwise a success. The accuracy shown is the inputs' average (a tap counts 100% when hit, 0% when missed).</t>
+  </si>
+  <si>
+    <t>Above the bar for 0.8 s: Miss, Good or Perfect!; a bar with a hold or several inputs adds its accuracy, e.g. Good 88%.</t>
+  </si>
+  <si>
+    <t>Zones separated by ';', each 'Tap a–b', 'Crit a–b' or 'Hold a–b', in seconds from the bar's start (for example 'Tap 0.35–0.65; Crit 0.45–0.55' or 'Hold 0.75–2.75', or a tap then a hold: 'Tap 0.20–0.60; Crit 0.35–0.45; Hold 1.00–3.75'). Dots or commas for decimals; '-' or '–' between the numbers.</t>
+  </si>
+  <si>
+    <t>Re-import the sheet (docs/ability-import.md). The import checks that every zone is inside its bar, that holds end 0.2–0.3 s before the bar, that crits sit inside a tap, that inputs don't overlap, and that the numbers read; it refuses the file otherwise.</t>
   </si>
 </sst>
 </file>
@@ -3819,10 +3831,10 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -11434,16 +11446,16 @@
       </c>
       <c r="T107" s="27"/>
       <c r="U107" s="27" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
       <c r="V107" s="27">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="W107" s="27" t="s">
-        <v>1013</v>
+        <v>1162</v>
       </c>
       <c r="X107" s="27" t="s">
-        <v>1014</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="108" spans="1:24" ht="42.75" x14ac:dyDescent="0.25">
@@ -11507,16 +11519,16 @@
       </c>
       <c r="T108" s="27"/>
       <c r="U108" s="27" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
       <c r="V108" s="27">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="W108" s="27" t="s">
-        <v>1015</v>
+        <v>1164</v>
       </c>
       <c r="X108" s="27" t="s">
-        <v>1016</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="109" spans="1:24" ht="28.5" x14ac:dyDescent="0.25">
@@ -12792,10 +12804,10 @@
         <v>1.2</v>
       </c>
       <c r="W127" s="32" t="s">
-        <v>1017</v>
+        <v>1013</v>
       </c>
       <c r="X127" s="32" t="s">
-        <v>1018</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="128" spans="1:24" ht="42.75" x14ac:dyDescent="0.25">
@@ -12868,7 +12880,7 @@
         <v>982</v>
       </c>
       <c r="X128" s="32" t="s">
-        <v>1019</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="129" spans="1:24" ht="42.75" x14ac:dyDescent="0.25">
@@ -14752,8 +14764,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44B4F233-3DD8-430F-97D9-38ED07DEBAB9}">
-  <dimension ref="A1:E66"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F2068AE-19BE-4F66-AA4F-E50C00860C0D}">
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -14764,850 +14776,874 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
-        <v>1020</v>
-      </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
+      <c r="A1" s="50" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
     </row>
     <row r="2" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="47" t="s">
-        <v>1021</v>
-      </c>
-      <c r="B2" s="48" t="s">
-        <v>1022</v>
-      </c>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
+        <v>1017</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
     </row>
     <row r="3" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>1023</v>
-      </c>
-      <c r="B3" s="48" t="s">
-        <v>1024</v>
-      </c>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
+        <v>1019</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
     </row>
     <row r="4" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
-        <v>1025</v>
-      </c>
-      <c r="B4" s="48" t="s">
-        <v>1026</v>
-      </c>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
+        <v>1021</v>
+      </c>
+      <c r="B4" s="49" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
-        <v>1027</v>
-      </c>
-      <c r="B5" s="48" t="s">
-        <v>1028</v>
-      </c>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-    </row>
-    <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1023</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+    </row>
+    <row r="6" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
-        <v>1029</v>
-      </c>
-      <c r="B6" s="48" t="s">
-        <v>1030</v>
-      </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-    </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1166</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+    </row>
+    <row r="7" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="47" t="s">
-        <v>1031</v>
-      </c>
-      <c r="B7" s="48" t="s">
-        <v>1032</v>
-      </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="46"/>
-      <c r="B8" s="46"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="46"/>
+        <v>1168</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+    </row>
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="47" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="49" t="s">
-        <v>1033</v>
-      </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
+      <c r="A9" s="46"/>
+      <c r="B9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B10" s="50"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="48" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B11" s="48" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C11" s="48" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>1031</v>
+      </c>
+      <c r="E11" s="48" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="47" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B12" s="47" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C12" s="47" t="s">
         <v>1034</v>
       </c>
-      <c r="B10" s="50" t="s">
+      <c r="D12" s="47" t="s">
         <v>1035</v>
       </c>
-      <c r="C10" s="50" t="s">
-        <v>1036</v>
-      </c>
-      <c r="D10" s="50" t="s">
-        <v>1037</v>
-      </c>
-      <c r="E10" s="50" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="47" t="s">
-        <v>1038</v>
-      </c>
-      <c r="B11" s="47" t="s">
-        <v>1039</v>
-      </c>
-      <c r="C11" s="47" t="s">
-        <v>1040</v>
-      </c>
-      <c r="D11" s="47" t="s">
-        <v>1041</v>
-      </c>
-      <c r="E11" s="47" t="s">
-        <v>1162</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
-        <v>1042</v>
-      </c>
-      <c r="B12" s="47" t="s">
-        <v>1043</v>
-      </c>
-      <c r="C12" s="47" t="s">
-        <v>1040</v>
-      </c>
-      <c r="D12" s="47" t="s">
-        <v>1044</v>
-      </c>
       <c r="E12" s="47" t="s">
-        <v>1045</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A13" s="47" t="s">
-        <v>1046</v>
+        <v>1036</v>
       </c>
       <c r="B13" s="47" t="s">
-        <v>1047</v>
+        <v>1037</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>1048</v>
+        <v>1034</v>
       </c>
       <c r="D13" s="47" t="s">
-        <v>1049</v>
+        <v>1038</v>
       </c>
       <c r="E13" s="47" t="s">
-        <v>1050</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A14" s="47" t="s">
-        <v>1051</v>
+        <v>1040</v>
       </c>
       <c r="B14" s="47" t="s">
-        <v>1052</v>
+        <v>1041</v>
       </c>
       <c r="C14" s="47" t="s">
-        <v>1053</v>
+        <v>1042</v>
       </c>
       <c r="D14" s="47" t="s">
-        <v>1054</v>
+        <v>1043</v>
       </c>
       <c r="E14" s="47" t="s">
-        <v>1162</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="46"/>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46"/>
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="47" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B15" s="47" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C15" s="47" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D15" s="47" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E15" s="47" t="s">
+        <v>1154</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="49" t="s">
-        <v>1055</v>
-      </c>
-      <c r="B16" s="49"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
+      <c r="A16" s="46"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="50" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B17" s="50"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="48" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B18" s="48" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D18" s="48" t="s">
+        <v>1051</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="47" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B19" s="47" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C19" s="47" t="s">
+        <v>1055</v>
+      </c>
+      <c r="D19" s="47" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E19" s="47" t="s">
         <v>1056</v>
       </c>
-      <c r="B17" s="50" t="s">
-        <v>1038</v>
-      </c>
-      <c r="C17" s="50" t="s">
-        <v>1046</v>
-      </c>
-      <c r="D17" s="50" t="s">
+    </row>
+    <row r="20" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="47" t="s">
         <v>1057</v>
       </c>
-      <c r="E17" s="50" t="s">
+      <c r="B20" s="47" t="s">
         <v>1058</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="47" t="s">
+      <c r="C20" s="47" t="s">
         <v>1059</v>
       </c>
-      <c r="B18" s="47" t="s">
+      <c r="D20" s="47" t="s">
         <v>1060</v>
       </c>
-      <c r="C18" s="47" t="s">
+      <c r="E20" s="47" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="47" t="s">
         <v>1061</v>
       </c>
-      <c r="D18" s="47" t="s">
-        <v>1163</v>
-      </c>
-      <c r="E18" s="47" t="s">
+      <c r="B21" s="47" t="s">
         <v>1062</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="47" t="s">
+      <c r="C21" s="47" t="s">
         <v>1063</v>
       </c>
-      <c r="B19" s="47" t="s">
+      <c r="D21" s="47" t="s">
+        <v>1156</v>
+      </c>
+      <c r="E21" s="47" t="s">
         <v>1064</v>
       </c>
-      <c r="C19" s="47" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="47" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+    </row>
+    <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="47" t="s">
         <v>1065</v>
       </c>
-      <c r="D19" s="47" t="s">
+      <c r="B23" s="49" t="s">
         <v>1066</v>
       </c>
-      <c r="E19" s="47" t="s">
-        <v>1062</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="47" t="s">
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+    </row>
+    <row r="24" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="47" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B24" s="49" t="s">
         <v>1067</v>
       </c>
-      <c r="B20" s="47" t="s">
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+    </row>
+    <row r="25" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="47" t="s">
         <v>1068</v>
       </c>
-      <c r="C20" s="47" t="s">
-        <v>1069</v>
-      </c>
-      <c r="D20" s="47" t="s">
-        <v>1164</v>
-      </c>
-      <c r="E20" s="47" t="s">
-        <v>1070</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="47" t="s">
-        <v>1071</v>
-      </c>
-      <c r="B21" s="48" t="s">
-        <v>1072</v>
-      </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-    </row>
-    <row r="22" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
-        <v>1058</v>
-      </c>
-      <c r="B22" s="48" t="s">
-        <v>1073</v>
-      </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-    </row>
-    <row r="23" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="47" t="s">
-        <v>1074</v>
-      </c>
-      <c r="B23" s="48" t="s">
-        <v>1165</v>
-      </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="49" t="s">
-        <v>1075</v>
-      </c>
-      <c r="B25" s="49"/>
+      <c r="B25" s="49" t="s">
+        <v>1172</v>
+      </c>
       <c r="C25" s="49"/>
       <c r="D25" s="49"/>
       <c r="E25" s="49"/>
     </row>
-    <row r="26" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="47" t="s">
-        <v>1076</v>
-      </c>
-      <c r="B26" s="48" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-    </row>
-    <row r="27" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
-        <v>1057</v>
-      </c>
-      <c r="B27" s="48" t="s">
-        <v>1078</v>
-      </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="46"/>
+      <c r="B26" s="46"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="50" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B27" s="50"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
     </row>
     <row r="28" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="47" t="s">
-        <v>1079</v>
-      </c>
-      <c r="B28" s="48" t="s">
-        <v>1080</v>
-      </c>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
-    </row>
-    <row r="29" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1070</v>
+      </c>
+      <c r="B28" s="49" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+    </row>
+    <row r="29" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="47" t="s">
-        <v>1081</v>
-      </c>
-      <c r="B29" s="48" t="s">
-        <v>1082</v>
-      </c>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-    </row>
-    <row r="30" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1051</v>
+      </c>
+      <c r="B29" s="49" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
+    </row>
+    <row r="30" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="47" t="s">
-        <v>1083</v>
-      </c>
-      <c r="B30" s="48" t="s">
-        <v>1084</v>
-      </c>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="48"/>
+        <v>1073</v>
+      </c>
+      <c r="B30" s="49" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
     </row>
     <row r="31" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="47" t="s">
-        <v>1085</v>
-      </c>
-      <c r="B31" s="48" t="s">
-        <v>1166</v>
-      </c>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="46"/>
-      <c r="B32" s="46"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="46"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="49" t="s">
-        <v>1086</v>
-      </c>
-      <c r="B33" s="49"/>
+        <v>1075</v>
+      </c>
+      <c r="B31" s="49" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
+    </row>
+    <row r="32" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="47" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B32" s="49" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+    </row>
+    <row r="33" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="47" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B33" s="49" t="s">
+        <v>1157</v>
+      </c>
       <c r="C33" s="49"/>
       <c r="D33" s="49"/>
       <c r="E33" s="49"/>
     </row>
-    <row r="34" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="47" t="s">
-        <v>1087</v>
-      </c>
-      <c r="B34" s="48" t="s">
-        <v>1088</v>
-      </c>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
-    </row>
-    <row r="35" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="47" t="s">
-        <v>1089</v>
-      </c>
-      <c r="B35" s="48" t="s">
-        <v>1090</v>
-      </c>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="46"/>
+      <c r="B34" s="46"/>
+      <c r="C34" s="46"/>
+      <c r="D34" s="46"/>
+      <c r="E34" s="46"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="50" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
     </row>
     <row r="36" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="47" t="s">
-        <v>1091</v>
-      </c>
-      <c r="B36" s="48" t="s">
-        <v>1092</v>
-      </c>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
-    </row>
-    <row r="37" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1081</v>
+      </c>
+      <c r="B36" s="49" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+    </row>
+    <row r="37" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="47" t="s">
-        <v>1093</v>
-      </c>
-      <c r="B37" s="48" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="46"/>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="49" t="s">
-        <v>1095</v>
-      </c>
-      <c r="B39" s="49"/>
+        <v>1083</v>
+      </c>
+      <c r="B37" s="49" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
+    </row>
+    <row r="38" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="47" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B38" s="49" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="49"/>
+    </row>
+    <row r="39" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="47" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B39" s="49" t="s">
+        <v>1088</v>
+      </c>
       <c r="C39" s="49"/>
       <c r="D39" s="49"/>
       <c r="E39" s="49"/>
     </row>
-    <row r="40" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="47" t="s">
-        <v>1096</v>
-      </c>
-      <c r="B40" s="48" t="s">
-        <v>1097</v>
-      </c>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-    </row>
-    <row r="41" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="47" t="s">
-        <v>1098</v>
-      </c>
-      <c r="B41" s="48" t="s">
-        <v>1099</v>
-      </c>
-      <c r="C41" s="48"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="46"/>
+      <c r="B40" s="46"/>
+      <c r="C40" s="46"/>
+      <c r="D40" s="46"/>
+      <c r="E40" s="46"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="50" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B41" s="50"/>
+      <c r="C41" s="50"/>
+      <c r="D41" s="50"/>
+      <c r="E41" s="50"/>
     </row>
     <row r="42" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="47" t="s">
-        <v>1100</v>
-      </c>
-      <c r="B42" s="48" t="s">
-        <v>1101</v>
-      </c>
-      <c r="C42" s="48"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="46"/>
-      <c r="B43" s="46"/>
-      <c r="C43" s="46"/>
-      <c r="D43" s="46"/>
-      <c r="E43" s="46"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="49" t="s">
-        <v>1102</v>
-      </c>
-      <c r="B44" s="49"/>
+        <v>1090</v>
+      </c>
+      <c r="B42" s="49" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49"/>
+      <c r="E42" s="49"/>
+    </row>
+    <row r="43" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="47" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B43" s="49" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C43" s="49"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="49"/>
+    </row>
+    <row r="44" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="47" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B44" s="49" t="s">
+        <v>1095</v>
+      </c>
       <c r="C44" s="49"/>
       <c r="D44" s="49"/>
       <c r="E44" s="49"/>
     </row>
-    <row r="45" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="47" t="s">
-        <v>963</v>
-      </c>
-      <c r="B45" s="48" t="s">
-        <v>1103</v>
-      </c>
-      <c r="C45" s="48"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="48"/>
-    </row>
-    <row r="46" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="47" t="s">
-        <v>964</v>
-      </c>
-      <c r="B46" s="48" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C46" s="48"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="46"/>
+      <c r="B45" s="46"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="50" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B46" s="50"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
+      <c r="E46" s="50"/>
     </row>
     <row r="47" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="47" t="s">
-        <v>965</v>
-      </c>
-      <c r="B47" s="48" t="s">
-        <v>1105</v>
-      </c>
-      <c r="C47" s="48"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
+        <v>963</v>
+      </c>
+      <c r="B47" s="49" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C47" s="49"/>
+      <c r="D47" s="49"/>
+      <c r="E47" s="49"/>
     </row>
     <row r="48" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="47" t="s">
+        <v>964</v>
+      </c>
+      <c r="B48" s="49" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C48" s="49"/>
+      <c r="D48" s="49"/>
+      <c r="E48" s="49"/>
+    </row>
+    <row r="49" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="47" t="s">
+        <v>965</v>
+      </c>
+      <c r="B49" s="49" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C49" s="49"/>
+      <c r="D49" s="49"/>
+      <c r="E49" s="49"/>
+    </row>
+    <row r="50" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="47" t="s">
         <v>966</v>
       </c>
-      <c r="B48" s="48" t="s">
-        <v>1106</v>
-      </c>
-      <c r="C48" s="48"/>
-      <c r="D48" s="48"/>
-      <c r="E48" s="48"/>
-    </row>
-    <row r="49" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="47" t="s">
-        <v>1107</v>
-      </c>
-      <c r="B49" s="48" t="s">
-        <v>1108</v>
-      </c>
-      <c r="C49" s="48"/>
-      <c r="D49" s="48"/>
-      <c r="E49" s="48"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="46"/>
-      <c r="B50" s="46"/>
-      <c r="C50" s="46"/>
-      <c r="D50" s="46"/>
-      <c r="E50" s="46"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="49" t="s">
-        <v>1109</v>
-      </c>
-      <c r="B51" s="49"/>
+      <c r="B50" s="49" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C50" s="49"/>
+      <c r="D50" s="49"/>
+      <c r="E50" s="49"/>
+    </row>
+    <row r="51" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="47" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B51" s="49" t="s">
+        <v>1174</v>
+      </c>
       <c r="C51" s="49"/>
       <c r="D51" s="49"/>
       <c r="E51" s="49"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="50" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B52" s="50" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C52" s="50" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D52" s="50" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E52" s="50" t="s">
-        <v>1113</v>
-      </c>
+      <c r="A52" s="46"/>
+      <c r="B52" s="46"/>
+      <c r="C52" s="46"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="47" t="s">
-        <v>1114</v>
-      </c>
-      <c r="B53" s="47" t="s">
-        <v>1167</v>
-      </c>
-      <c r="C53" s="47" t="s">
-        <v>1115</v>
-      </c>
-      <c r="D53" s="47" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E53" s="47" t="s">
-        <v>1116</v>
-      </c>
+      <c r="A53" s="50" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B53" s="50"/>
+      <c r="C53" s="50"/>
+      <c r="D53" s="50"/>
+      <c r="E53" s="50"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="47" t="s">
-        <v>1117</v>
-      </c>
-      <c r="B54" s="47" t="s">
-        <v>1168</v>
-      </c>
-      <c r="C54" s="47" t="s">
-        <v>1118</v>
-      </c>
-      <c r="D54" s="47" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E54" s="47" t="s">
-        <v>1119</v>
+      <c r="A54" s="48" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B54" s="48" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C54" s="48" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D54" s="48" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E54" s="48" t="s">
+        <v>1105</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="47" t="s">
-        <v>1120</v>
+        <v>1106</v>
       </c>
       <c r="B55" s="47" t="s">
-        <v>1169</v>
+        <v>1158</v>
       </c>
       <c r="C55" s="47" t="s">
-        <v>1121</v>
+        <v>1107</v>
       </c>
       <c r="D55" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E55" s="47" t="s">
-        <v>1122</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="47" t="s">
-        <v>1123</v>
+        <v>1109</v>
       </c>
       <c r="B56" s="47" t="s">
-        <v>1124</v>
+        <v>1159</v>
       </c>
       <c r="C56" s="47" t="s">
-        <v>1125</v>
+        <v>1110</v>
       </c>
       <c r="D56" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E56" s="47" t="s">
-        <v>1126</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="47" t="s">
-        <v>1127</v>
+        <v>1112</v>
       </c>
       <c r="B57" s="47" t="s">
-        <v>1128</v>
+        <v>1160</v>
       </c>
       <c r="C57" s="47" t="s">
-        <v>1129</v>
+        <v>1113</v>
       </c>
       <c r="D57" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E57" s="47" t="s">
-        <v>1130</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A58" s="47" t="s">
-        <v>1131</v>
+        <v>1115</v>
       </c>
       <c r="B58" s="47" t="s">
-        <v>1132</v>
+        <v>1116</v>
       </c>
       <c r="C58" s="47" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="D58" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E58" s="47" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A59" s="47" t="s">
-        <v>1135</v>
+        <v>1119</v>
       </c>
       <c r="B59" s="47" t="s">
-        <v>1136</v>
+        <v>1120</v>
       </c>
       <c r="C59" s="47" t="s">
-        <v>1137</v>
+        <v>1121</v>
       </c>
       <c r="D59" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E59" s="47" t="s">
-        <v>1138</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A60" s="47" t="s">
-        <v>1139</v>
+        <v>1123</v>
       </c>
       <c r="B60" s="47" t="s">
-        <v>1140</v>
+        <v>1124</v>
       </c>
       <c r="C60" s="47" t="s">
-        <v>1141</v>
+        <v>1125</v>
       </c>
       <c r="D60" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E60" s="47" t="s">
-        <v>1142</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
-        <v>1143</v>
+        <v>1127</v>
       </c>
       <c r="B61" s="47" t="s">
-        <v>1170</v>
+        <v>1128</v>
       </c>
       <c r="C61" s="47" t="s">
-        <v>1144</v>
+        <v>1129</v>
       </c>
       <c r="D61" s="47" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="E61" s="47" t="s">
-        <v>1145</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="47" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B62" s="47" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C62" s="47" t="s">
+        <v>1133</v>
+      </c>
+      <c r="D62" s="47" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E62" s="47" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="47" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B63" s="47" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C63" s="47" t="s">
+        <v>1136</v>
+      </c>
+      <c r="D63" s="47" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E63" s="47" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="47" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B64" s="47" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C64" s="47" t="s">
+        <v>1140</v>
+      </c>
+      <c r="D64" s="47" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E64" s="47" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="47" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B65" s="47" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C65" s="47" t="s">
+        <v>1144</v>
+      </c>
+      <c r="D65" s="47" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E65" s="47" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="47" t="s">
         <v>1146</v>
       </c>
-      <c r="B62" s="47" t="s">
+      <c r="B66" s="47" t="s">
         <v>1147</v>
       </c>
-      <c r="C62" s="47" t="s">
+      <c r="C66" s="47" t="s">
         <v>1148</v>
       </c>
-      <c r="D62" s="47" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E62" s="47" t="s">
+      <c r="D66" s="47" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E66" s="47" t="s">
         <v>1149</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="47" t="s">
+    <row r="67" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="47" t="s">
         <v>1150</v>
       </c>
-      <c r="B63" s="47" t="s">
+      <c r="B67" s="47" t="s">
         <v>1151</v>
       </c>
-      <c r="C63" s="47" t="s">
+      <c r="C67" s="47" t="s">
         <v>1152</v>
       </c>
-      <c r="D63" s="47" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E63" s="47" t="s">
+      <c r="D67" s="47" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E67" s="47" t="s">
         <v>1153</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="47" t="s">
-        <v>1154</v>
-      </c>
-      <c r="B64" s="47" t="s">
-        <v>1155</v>
-      </c>
-      <c r="C64" s="47" t="s">
-        <v>1156</v>
-      </c>
-      <c r="D64" s="47" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E64" s="47" t="s">
-        <v>1157</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="47" t="s">
-        <v>1158</v>
-      </c>
-      <c r="B65" s="47" t="s">
-        <v>1159</v>
-      </c>
-      <c r="C65" s="47" t="s">
-        <v>1160</v>
-      </c>
-      <c r="D65" s="47" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E65" s="47" t="s">
-        <v>1161</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="46"/>
-      <c r="B66" s="46"/>
-      <c r="C66" s="46"/>
-      <c r="D66" s="46"/>
-      <c r="E66" s="46"/>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="46"/>
+      <c r="B68" s="46"/>
+      <c r="C68" s="46"/>
+      <c r="D68" s="46"/>
+      <c r="E68" s="46"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="B46:E46"/>
+  <mergeCells count="37">
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A46:E46"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="B49:E49"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="A41:E41"/>
     <mergeCell ref="B42:E42"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B44:E44"/>
     <mergeCell ref="B31:E31"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B36:E36"/>
     <mergeCell ref="B37:E37"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="A27:E27"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="A1:E1"/>

</xml_diff>